<commit_message>
data: renumber KHTN 8 YCCD per topic (grade-7 rule); approve source flags for 7 and 9
- Outcome_YCCD_KHTN_8.xlsx: YCCD numbers restart at 1 inside each branch
  topic, in source row order (56 cells; e.g. H.2.4 -> H.2.1, the duplicate
  S.18.1 -> S.18.2). Statement text unchanged, no source flags left, so
  grade 8 imports without --renumber-duplicates.
- build-khtn-lesson-seed: default OUTCOME_DIR is the repo workbook copy so
  seed ordinals match what the server loads; khtn8-lessons.json and the
  review doc regenerated (coverage unchanged).
- v6671-lesson-seed test: grade 8 check has no duplicates/risky rows, all
  grades import with renumbered = [], DB ordinals H.2 = 1..8, S.18 = 1..5.
- Ubuntu guide section 10 A1: grades 7 and 9 --accept-source-warnings
  approved by the owner; grade 8 needs no flag; anything else -> STOP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/src/db/seed-data/curriculum/Outcome_YCCD_KHTN_8.xlsx
+++ b/backend/src/db/seed-data/curriculum/Outcome_YCCD_KHTN_8.xlsx
@@ -478,7 +478,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C9" t="str">
-        <v>4. Nêu được khái niệm sự biến đổi vật lí, biến đổi hoá học.</v>
+        <v>1. Nêu được khái niệm sự biến đổi vật lí, biến đổi hoá học.</v>
       </c>
       <c r="D9" t="str">
         <v>43</v>
@@ -492,7 +492,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C10" t="str">
-        <v>5. Phân biệt được sự biến đổi vật lí, biến đổi hoá học. Đưa ra được ví dụ về sự biến đổi vật lí và sự biến đổi hoá học.</v>
+        <v>2. Phân biệt được sự biến đổi vật lí, biến đổi hoá học. Đưa ra được ví dụ về sự biến đổi vật lí và sự biến đổi hoá học.</v>
       </c>
       <c r="D10" t="str">
         <v>43</v>
@@ -506,7 +506,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C11" t="str">
-        <v>6. Tiến hành được một số thí nghiệm về sự biến đổi vật lí và biến đổi hoá học.</v>
+        <v>3. Tiến hành được một số thí nghiệm về sự biến đổi vật lí và biến đổi hoá học.</v>
       </c>
       <c r="D11" t="str">
         <v>43</v>
@@ -520,7 +520,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C12" t="str">
-        <v>7. Nêu được khái niệm phản ứng hoá học, chất đầu và sản phẩm.</v>
+        <v>4. Nêu được khái niệm phản ứng hoá học, chất đầu và sản phẩm.</v>
       </c>
       <c r="D12" t="str">
         <v>43</v>
@@ -534,7 +534,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C13" t="str">
-        <v>8. Nêu được sự sắp xếp khác nhau của các nguyên tử trong phân tử chất đầu và sản phẩm</v>
+        <v>5. Nêu được sự sắp xếp khác nhau của các nguyên tử trong phân tử chất đầu và sản phẩm</v>
       </c>
       <c r="D13" t="str">
         <v>43</v>
@@ -548,7 +548,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C14" t="str">
-        <v>9. Chỉ ra được một số dấu hiệu chứng tỏ có phản ứng hoá học xảy ra.</v>
+        <v>6. Chỉ ra được một số dấu hiệu chứng tỏ có phản ứng hoá học xảy ra.</v>
       </c>
       <c r="D14" t="str">
         <v>43</v>
@@ -562,7 +562,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C15" t="str">
-        <v>10. Nêu được khái niệm và đưa ra được ví dụ minh hoạ về phản ứng toả nhiệt, thu nhiệt.</v>
+        <v>7. Nêu được khái niệm và đưa ra được ví dụ minh hoạ về phản ứng toả nhiệt, thu nhiệt.</v>
       </c>
       <c r="D15" t="str">
         <v>43</v>
@@ -576,7 +576,7 @@
         <v>2.Phản ứng hóa học</v>
       </c>
       <c r="C16" t="str">
-        <v>11. Trình bày được các ứng dụng phổ biến của phản ứng toả nhiệt (đốt cháy than, xăng, dầu).</v>
+        <v>8. Trình bày được các ứng dụng phổ biến của phản ứng toả nhiệt (đốt cháy than, xăng, dầu).</v>
       </c>
       <c r="D16" t="str">
         <v>43</v>
@@ -590,7 +590,7 @@
         <v>3.Định luật bảo toàn khối lượng và phương trình hóa học</v>
       </c>
       <c r="C17" t="str">
-        <v>12. Tiến hành được thí nghiệm để chứng minh: Trong phản ứng hoá học, khối lượng được bảo toàn.</v>
+        <v>1. Tiến hành được thí nghiệm để chứng minh: Trong phản ứng hoá học, khối lượng được bảo toàn.</v>
       </c>
       <c r="D17" t="str">
         <v>43</v>
@@ -604,7 +604,7 @@
         <v>3.Định luật bảo toàn khối lượng và phương trình hóa học</v>
       </c>
       <c r="C18" t="str">
-        <v>13. Phát biểu được định luật bảo toàn khối lượng.</v>
+        <v>2. Phát biểu được định luật bảo toàn khối lượng.</v>
       </c>
       <c r="D18" t="str">
         <v>43</v>
@@ -618,7 +618,7 @@
         <v>3.Định luật bảo toàn khối lượng và phương trình hóa học</v>
       </c>
       <c r="C19" t="str">
-        <v>14. Nêu được khái niệm phương trình hoá học và các bước lập phương trình hoá học.</v>
+        <v>3. Nêu được khái niệm phương trình hoá học và các bước lập phương trình hoá học.</v>
       </c>
       <c r="D19" t="str">
         <v>43–44</v>
@@ -632,7 +632,7 @@
         <v>3.Định luật bảo toàn khối lượng và phương trình hóa học</v>
       </c>
       <c r="C20" t="str">
-        <v>15. Trình bày được ý nghĩa của phương trình hoá học.</v>
+        <v>4. Trình bày được ý nghĩa của phương trình hoá học.</v>
       </c>
       <c r="D20" t="str">
         <v>43–44</v>
@@ -646,7 +646,7 @@
         <v>3.Định luật bảo toàn khối lượng và phương trình hóa học</v>
       </c>
       <c r="C21" t="str">
-        <v>16. Lập được sơ đồ phản ứng hoá học dạng chữ và phương trình hoá học (dùng công thức hoá học) của một số phản ứng hoá học cụ thể.</v>
+        <v>5. Lập được sơ đồ phản ứng hoá học dạng chữ và phương trình hoá học (dùng công thức hoá học) của một số phản ứng hoá học cụ thể.</v>
       </c>
       <c r="D21" t="str">
         <v>43–44</v>
@@ -660,7 +660,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C22" t="str">
-        <v>17. Nêu được khái niệm về mol (nguyên tử, phân tử).</v>
+        <v>1. Nêu được khái niệm về mol (nguyên tử, phân tử).</v>
       </c>
       <c r="D22" t="str">
         <v>44</v>
@@ -674,7 +674,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C23" t="str">
-        <v>18. Tính được khối lượng mol (M); Chuyển đổi được giữa số mol (n) và khối lượng (m)</v>
+        <v>2. Tính được khối lượng mol (M); Chuyển đổi được giữa số mol (n) và khối lượng (m)</v>
       </c>
       <c r="D23" t="str">
         <v>44</v>
@@ -688,7 +688,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C24" t="str">
-        <v>19. Nêu được khái niệm tỉ khối, viết được công thức tính tỉ khối của chất khí.</v>
+        <v>3. Nêu được khái niệm tỉ khối, viết được công thức tính tỉ khối của chất khí.</v>
       </c>
       <c r="D24" t="str">
         <v>44</v>
@@ -702,7 +702,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C25" t="str">
-        <v>20. So sánh được chất khí này nặng hay nhẹ hơn chất khí khác dựa vào công thức tính tỉ khối.</v>
+        <v>4. So sánh được chất khí này nặng hay nhẹ hơn chất khí khác dựa vào công thức tính tỉ khối.</v>
       </c>
       <c r="D25" t="str">
         <v>44</v>
@@ -716,7 +716,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C26" t="str">
-        <v>21. Nêu được khái niệm thể tích mol của chất khí ở áp suất 1 bar và 25 °C.</v>
+        <v>5. Nêu được khái niệm thể tích mol của chất khí ở áp suất 1 bar và 25 °C.</v>
       </c>
       <c r="D26" t="str">
         <v>44</v>
@@ -730,7 +730,7 @@
         <v>4.Mol và tỉ khối chất khí</v>
       </c>
       <c r="C27" t="str">
-        <v>22. Sử dụng được công thức n (mol) = V (L) / 24,79 (L/mol) để chuyển đổi giữa số mol và thể tích chất khí ở điều kiện chuẩn: áp suất 1 bar và 25 °C.</v>
+        <v>6. Sử dụng được công thức n (mol) = V (L) / 24,79 (L/mol) để chuyển đổi giữa số mol và thể tích chất khí ở điều kiện chuẩn: áp suất 1 bar và 25 °C.</v>
       </c>
       <c r="D27" t="str">
         <v>44</v>
@@ -744,7 +744,7 @@
         <v>5.Tính theo phương trình hóa học</v>
       </c>
       <c r="C28" t="str">
-        <v>23. Tính được lượng chất trong phương trình hóa học theo số mol, khối lượng hoặc thể tích ở điều kiện 1 bar và 25 °C.</v>
+        <v>1. Tính được lượng chất trong phương trình hóa học theo số mol, khối lượng hoặc thể tích ở điều kiện 1 bar và 25 °C.</v>
       </c>
       <c r="D28" t="str">
         <v>44</v>
@@ -758,7 +758,7 @@
         <v>5.Tính theo phương trình hóa học</v>
       </c>
       <c r="C29" t="str">
-        <v>24. Nêu được khái niệm hiệu suất của phản ứng và tính được hiệu suất của một phản ứng dựa vào lượng sản phẩm thu được theo lí thuyết và lượng sản phẩm thu được theo thực tế.</v>
+        <v>2. Nêu được khái niệm hiệu suất của phản ứng và tính được hiệu suất của một phản ứng dựa vào lượng sản phẩm thu được theo lí thuyết và lượng sản phẩm thu được theo thực tế.</v>
       </c>
       <c r="D29" t="str">
         <v>44</v>
@@ -772,7 +772,7 @@
         <v>6.Dung dịch và nồng độ</v>
       </c>
       <c r="C30" t="str">
-        <v>25. Nêu được dung dịch là hỗn hợp lỏng đồng nhất của các chất đã tan trong nhau.</v>
+        <v>1. Nêu được dung dịch là hỗn hợp lỏng đồng nhất của các chất đã tan trong nhau.</v>
       </c>
       <c r="D30" t="str">
         <v>44</v>
@@ -786,7 +786,7 @@
         <v>6.Dung dịch và nồng độ</v>
       </c>
       <c r="C31" t="str">
-        <v>26. Nêu được định nghĩa độ tan của một chất trong nước, nồng độ phần trăm, nồng độ mol.</v>
+        <v>2. Nêu được định nghĩa độ tan của một chất trong nước, nồng độ phần trăm, nồng độ mol.</v>
       </c>
       <c r="D31" t="str">
         <v>44</v>
@@ -800,7 +800,7 @@
         <v>6.Dung dịch và nồng độ</v>
       </c>
       <c r="C32" t="str">
-        <v>27. Tính được độ tan, nồng độ phần trăm; nồng độ mol theo công thức.</v>
+        <v>3. Tính được độ tan, nồng độ phần trăm; nồng độ mol theo công thức.</v>
       </c>
       <c r="D32" t="str">
         <v>44</v>
@@ -814,7 +814,7 @@
         <v>6.Dung dịch và nồng độ</v>
       </c>
       <c r="C33" t="str">
-        <v>28. Tiến hành được thí nghiệm pha một dung dịch theo một nồng độ cho trước.</v>
+        <v>4. Tiến hành được thí nghiệm pha một dung dịch theo một nồng độ cho trước.</v>
       </c>
       <c r="D33" t="str">
         <v>44</v>
@@ -828,7 +828,7 @@
         <v>7.Tốc độ phản ứng</v>
       </c>
       <c r="C34" t="str">
-        <v>29. Nêu được khái niệm về tốc độ phản ứng (chỉ mức độ nhanh hay chậm của phản ứng hoá học).</v>
+        <v>1. Nêu được khái niệm về tốc độ phản ứng (chỉ mức độ nhanh hay chậm của phản ứng hoá học).</v>
       </c>
       <c r="D34" t="str">
         <v>44–45</v>
@@ -842,7 +842,7 @@
         <v>7.Tốc độ phản ứng</v>
       </c>
       <c r="C35" t="str">
-        <v>30. Trình bày được một số yếu tố ảnh hưởng đến tốc độ phản ứng và nêu được một số ứng dụng thực tế.</v>
+        <v>2. Trình bày được một số yếu tố ảnh hưởng đến tốc độ phản ứng và nêu được một số ứng dụng thực tế.</v>
       </c>
       <c r="D35" t="str">
         <v>44–45</v>
@@ -856,7 +856,7 @@
         <v>7.Tốc độ phản ứng</v>
       </c>
       <c r="C36" t="str" xml:space="preserve">
-        <v xml:space="preserve">31. Tiến hành được thí nghiệm và quan sát thực tiễn:
+        <v xml:space="preserve">3. Tiến hành được thí nghiệm và quan sát thực tiễn:
 + So sánh được tốc độ một số phản ứng hoá học;
 + Nêu được các yếu tố làm thay đổi tốc độ phản ứng;
 + Nêu được khái niệm về chất xúc tác.</v>
@@ -873,7 +873,7 @@
         <v>8.Acid</v>
       </c>
       <c r="C37" t="str">
-        <v>32. Nêu được khái niệm acid (tạo ra ion H+).</v>
+        <v>1. Nêu được khái niệm acid (tạo ra ion H+).</v>
       </c>
       <c r="D37" t="str">
         <v>45</v>
@@ -887,7 +887,7 @@
         <v>8.Acid</v>
       </c>
       <c r="C38" t="str">
-        <v>33. Tiến hành được thí nghiệm của hydrochloric acid (làm đổi màu chất chỉ thị; phản ứng với kim loại), nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất của acid.</v>
+        <v>2. Tiến hành được thí nghiệm của hydrochloric acid (làm đổi màu chất chỉ thị; phản ứng với kim loại), nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất của acid.</v>
       </c>
       <c r="D38" t="str">
         <v>45</v>
@@ -901,7 +901,7 @@
         <v>8.Acid</v>
       </c>
       <c r="C39" t="str">
-        <v>34. Trình bày được một số ứng dụng của một số acid thông dụng (HCl, H₂SO₄, CH₃COOH).</v>
+        <v>3. Trình bày được một số ứng dụng của một số acid thông dụng (HCl, H₂SO₄, CH₃COOH).</v>
       </c>
       <c r="D39" t="str">
         <v>45</v>
@@ -915,7 +915,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C40" t="str">
-        <v>35. Nêu được khái niệm base (tạo ra ion OH–).</v>
+        <v>1. Nêu được khái niệm base (tạo ra ion OH–).</v>
       </c>
       <c r="D40" t="str">
         <v>45</v>
@@ -929,7 +929,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C41" t="str">
-        <v>36. Nêu được kiềm là các hydroxide tan tốt trong nước.</v>
+        <v>2. Nêu được kiềm là các hydroxide tan tốt trong nước.</v>
       </c>
       <c r="D41" t="str">
         <v>45</v>
@@ -943,7 +943,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C42" t="str">
-        <v>37. Tiến hành được thí nghiệm base là làm đổi màu chất chỉ thị, phản ứng với acid tạo muối, nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất của base.</v>
+        <v>3. Tiến hành được thí nghiệm base là làm đổi màu chất chỉ thị, phản ứng với acid tạo muối, nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất của base.</v>
       </c>
       <c r="D42" t="str">
         <v>45</v>
@@ -957,7 +957,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C43" t="str">
-        <v>38. Tra được bảng tính tan để biết một hydroxide cụ thể thuộc loại kiềm hoặc base không tan.</v>
+        <v>4. Tra được bảng tính tan để biết một hydroxide cụ thể thuộc loại kiềm hoặc base không tan.</v>
       </c>
       <c r="D43" t="str">
         <v>45</v>
@@ -971,7 +971,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C44" t="str">
-        <v>39. Nêu được thang pH, sử dụng pH để đánh giá độ acid - base của dung dịch.</v>
+        <v>5. Nêu được thang pH, sử dụng pH để đánh giá độ acid - base của dung dịch.</v>
       </c>
       <c r="D44" t="str">
         <v>45–46</v>
@@ -985,7 +985,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C45" t="str">
-        <v>40. Tiến hành được một số thí nghiệm đo pH (bằng giấy chỉ thị) một số loại thực phẩm (đồ uống, hoa quả,...).</v>
+        <v>6. Tiến hành được một số thí nghiệm đo pH (bằng giấy chỉ thị) một số loại thực phẩm (đồ uống, hoa quả,...).</v>
       </c>
       <c r="D45" t="str">
         <v>45–46</v>
@@ -999,7 +999,7 @@
         <v>9.Base. Thang pH</v>
       </c>
       <c r="C46" t="str">
-        <v>41. Liên hệ được pH trong dạ dày, trong máu, trong nước mưa, đất.</v>
+        <v>7. Liên hệ được pH trong dạ dày, trong máu, trong nước mưa, đất.</v>
       </c>
       <c r="D46" t="str">
         <v>45–46</v>
@@ -1013,7 +1013,7 @@
         <v>10.Oxide</v>
       </c>
       <c r="C47" t="str">
-        <v>42. Nêu được khái niệm oxide là hợp chất của oxygen với một nguyên tố khác.</v>
+        <v>1. Nêu được khái niệm oxide là hợp chất của oxygen với một nguyên tố khác.</v>
       </c>
       <c r="D47" t="str">
         <v>46</v>
@@ -1027,7 +1027,7 @@
         <v>10.Oxide</v>
       </c>
       <c r="C48" t="str">
-        <v>43. Viết được phương trình hoá học tạo oxide từ kim loại/phi kim với oxygen.</v>
+        <v>2. Viết được phương trình hoá học tạo oxide từ kim loại/phi kim với oxygen.</v>
       </c>
       <c r="D48" t="str">
         <v>46</v>
@@ -1041,7 +1041,7 @@
         <v>10.Oxide</v>
       </c>
       <c r="C49" t="str">
-        <v>44. Phân loại được các oxide theo khả năng phản ứng với acid/base (oxide acid, oxide base, oxide lưỡng tính, oxide trung tính).</v>
+        <v>3. Phân loại được các oxide theo khả năng phản ứng với acid/base (oxide acid, oxide base, oxide lưỡng tính, oxide trung tính).</v>
       </c>
       <c r="D49" t="str">
         <v>46</v>
@@ -1055,7 +1055,7 @@
         <v>10.Oxide</v>
       </c>
       <c r="C50" t="str">
-        <v>45. Tiến hành được thí nghiệm oxide kim loại phản ứng với acid; oxide phi kim phản ứng với base; nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất hoá học của oxide.</v>
+        <v>4. Tiến hành được thí nghiệm oxide kim loại phản ứng với acid; oxide phi kim phản ứng với base; nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra nhận xét về tính chất hoá học của oxide.</v>
       </c>
       <c r="D50" t="str">
         <v>46</v>
@@ -1069,7 +1069,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C51" t="str">
-        <v>46. Nêu được khái niệm về muối (các muối thông thường là hợp chất được hình thành từ sự thay thế ion H+ của acid bởi ion kim loại hoặc ion NH₄⁺).</v>
+        <v>1. Nêu được khái niệm về muối (các muối thông thường là hợp chất được hình thành từ sự thay thế ion H+ của acid bởi ion kim loại hoặc ion NH₄⁺).</v>
       </c>
       <c r="D51" t="str">
         <v>46</v>
@@ -1083,7 +1083,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C52" t="str">
-        <v>47. Chỉ ra được một số muối tan và muối không tan từ bảng tính tan.</v>
+        <v>2. Chỉ ra được một số muối tan và muối không tan từ bảng tính tan.</v>
       </c>
       <c r="D52" t="str">
         <v>46</v>
@@ -1097,7 +1097,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C53" t="str">
-        <v>48. Trình bày được một số phương pháp điều chế muối.</v>
+        <v>3. Trình bày được một số phương pháp điều chế muối.</v>
       </c>
       <c r="D53" t="str">
         <v>46</v>
@@ -1111,7 +1111,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C54" t="str">
-        <v>49. Đọc được tên một số loại muối thông dụng.</v>
+        <v>4. Đọc được tên một số loại muối thông dụng.</v>
       </c>
       <c r="D54" t="str">
         <v>46</v>
@@ -1125,7 +1125,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C55" t="str">
-        <v>50. Tiến hành được thí nghiệm muối phản ứng với kim loại, với acid, với base, với muối; nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra kết luận về tính chất hoá học của muối.</v>
+        <v>5. Tiến hành được thí nghiệm muối phản ứng với kim loại, với acid, với base, với muối; nêu và giải thích được hiện tượng xảy ra trong thí nghiệm (viết phương trình hoá học) và rút ra kết luận về tính chất hoá học của muối.</v>
       </c>
       <c r="D55" t="str">
         <v>46</v>
@@ -1139,7 +1139,7 @@
         <v>11.Muối</v>
       </c>
       <c r="C56" t="str">
-        <v>51. Trình bày được mối quan hệ giữa acid, base, oxide và muối; rút ra được kết luận về tính chất hoá học của acid, base, oxide.</v>
+        <v>6. Trình bày được mối quan hệ giữa acid, base, oxide và muối; rút ra được kết luận về tính chất hoá học của acid, base, oxide.</v>
       </c>
       <c r="D56" t="str">
         <v>46</v>
@@ -1153,7 +1153,7 @@
         <v>12.Phân bón hóa học</v>
       </c>
       <c r="C57" t="str">
-        <v>52. Trình bày được vai trò của phân bón (một trong những nguồn bổ sung một số nguyên tố: đa lượng, trung lượng, vi lượng dưới dạng vô cơ và hữu cơ) cho đất, cây trồng.</v>
+        <v>1. Trình bày được vai trò của phân bón (một trong những nguồn bổ sung một số nguyên tố: đa lượng, trung lượng, vi lượng dưới dạng vô cơ và hữu cơ) cho đất, cây trồng.</v>
       </c>
       <c r="D57" t="str">
         <v>46–47</v>
@@ -1167,7 +1167,7 @@
         <v>12.Phân bón hóa học</v>
       </c>
       <c r="C58" t="str">
-        <v>53. Nêu được thành phần và tác dụng cơ bản của một số loại phân bón hoá học đối với cây trồng (phân đạm, phân lân, phân kali, phân N–P–K).</v>
+        <v>2. Nêu được thành phần và tác dụng cơ bản của một số loại phân bón hoá học đối với cây trồng (phân đạm, phân lân, phân kali, phân N–P–K).</v>
       </c>
       <c r="D58" t="str">
         <v>46–47</v>
@@ -1181,7 +1181,7 @@
         <v>12.Phân bón hóa học</v>
       </c>
       <c r="C59" t="str">
-        <v>54. Trình bày được ảnh hưởng của việc sử dụng phân bón hoá học (không đúng cách, không đúng liều lượng) đến môi trường của đất, nước và sức khoẻ của con người.</v>
+        <v>3. Trình bày được ảnh hưởng của việc sử dụng phân bón hoá học (không đúng cách, không đúng liều lượng) đến môi trường của đất, nước và sức khoẻ của con người.</v>
       </c>
       <c r="D59" t="str">
         <v>46–47</v>
@@ -1195,7 +1195,7 @@
         <v>12.Phân bón hóa học</v>
       </c>
       <c r="C60" t="str">
-        <v>55. Đề xuất được biện pháp giảm thiểu ô nhiễm của phân bón.</v>
+        <v>4. Đề xuất được biện pháp giảm thiểu ô nhiễm của phân bón.</v>
       </c>
       <c r="D60" t="str">
         <v>46–47</v>
@@ -3102,7 +3102,7 @@
         <v>18.Bảo vệ môi trường</v>
       </c>
       <c r="C196" t="str">
-        <v>1. Nêu được khái niệm ô nhiễm môi trường. Trình bày được sơ lược về một số nguyên nhân gây ô nhiễm môi trường (ô nhiễm do chất thải sinh hoạt và công nghiệp, ô nhiễm hoá chất bảo vệ thực vật, ô nhiễm phóng xạ, ô nhiễm do sinh vật gây bệnh) và biện pháp hạn chế ô nhiễm môi trường.</v>
+        <v>2. Nêu được khái niệm ô nhiễm môi trường. Trình bày được sơ lược về một số nguyên nhân gây ô nhiễm môi trường (ô nhiễm do chất thải sinh hoạt và công nghiệp, ô nhiễm hoá chất bảo vệ thực vật, ô nhiễm phóng xạ, ô nhiễm do sinh vật gây bệnh) và biện pháp hạn chế ô nhiễm môi trường.</v>
       </c>
       <c r="D196" t="str">
         <v>59</v>
@@ -3116,7 +3116,7 @@
         <v>18.Bảo vệ môi trường</v>
       </c>
       <c r="C197" t="str">
-        <v>2. Trình bày được sự cần thiết phải bảo vệ động vật hoang dã, nhất là những loài có nguy cơ bị tuyệt chủng cần được bảo vệ theo Công ước quốc tế về buôn bán các loài động, thực vật hoang dã (CITES) (ví dụ như các loài voi, tê giác, hổ, sếu đầu đỏ và các loài linh trưởng,…).</v>
+        <v>3. Trình bày được sự cần thiết phải bảo vệ động vật hoang dã, nhất là những loài có nguy cơ bị tuyệt chủng cần được bảo vệ theo Công ước quốc tế về buôn bán các loài động, thực vật hoang dã (CITES) (ví dụ như các loài voi, tê giác, hổ, sếu đầu đỏ và các loài linh trưởng,…).</v>
       </c>
       <c r="D197" t="str">
         <v>59</v>
@@ -3130,7 +3130,7 @@
         <v>18.Bảo vệ môi trường</v>
       </c>
       <c r="C198" t="str">
-        <v>3. Nêu được khái niệm khái quát về biến đổi khí hậu và một số biện pháp chủ yếu nhằm thích ứng với biến đổi khí hậu.</v>
+        <v>4. Nêu được khái niệm khái quát về biến đổi khí hậu và một số biện pháp chủ yếu nhằm thích ứng với biến đổi khí hậu.</v>
       </c>
       <c r="D198" t="str">
         <v>59</v>
@@ -3144,7 +3144,7 @@
         <v>18.Bảo vệ môi trường</v>
       </c>
       <c r="C199" t="str">
-        <v>4. Điều tra được hiện trạng ô nhiễm môi trường ở địa phương.</v>
+        <v>5. Điều tra được hiện trạng ô nhiễm môi trường ở địa phương.</v>
       </c>
       <c r="D199" t="str">
         <v>59</v>

</xml_diff>